<commit_message>
Date: 12 Apr 2026
</commit_message>
<xml_diff>
--- a/MyAutomationProject/ExcelFiles/LoginData.xlsx
+++ b/MyAutomationProject/ExcelFiles/LoginData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AViIT\Demos\Selenium_16\MyAutomationProject\ExcelFiles\"/>
     </mc:Choice>
@@ -16,7 +16,7 @@
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="15">
   <si>
     <t>User Name</t>
   </si>
@@ -44,9 +44,6 @@
     <t>standard_user</t>
   </si>
   <si>
-    <t>locked_out_user</t>
-  </si>
-  <si>
     <t>kamini</t>
   </si>
   <si>
@@ -63,19 +60,34 @@
   </si>
   <si>
     <t>pravin</t>
+  </si>
+  <si>
+    <t>error_user</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -98,9 +110,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -384,7 +397,7 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -398,7 +411,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -409,80 +422,80 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
+      <c r="A4" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Date: 18 Apr 2026
</commit_message>
<xml_diff>
--- a/MyAutomationProject/ExcelFiles/LoginData.xlsx
+++ b/MyAutomationProject/ExcelFiles/LoginData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="17">
   <si>
     <t>User Name</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>Fail</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username and password do not match any user in this service</t>
   </si>
 </sst>
 </file>
@@ -425,7 +431,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -439,7 +445,7 @@
         <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -453,7 +459,7 @@
         <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -467,7 +473,7 @@
         <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -481,7 +487,7 @@
         <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -495,7 +501,7 @@
         <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>